<commit_message>
Correção gráficos do resíduo de Cox-Snell
</commit_message>
<xml_diff>
--- a/banco/turnover.xlsx
+++ b/banco/turnover.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funcapes-my.sharepoint.com/personal/lucas_alves_capes_gov_br/Documents/Área de Trabalho/UnB/Análise de Sobrevivência/Trabalho Sobrevivência/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/193a817bb0670a4b/Área de Trabalho/Projetos R/Sobrevivência/Turnover-Sobrevivencia/banco/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="32" documentId="8_{41879A0E-1429-4A20-A9DC-82B962858FE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1982131B-D120-4FC3-83B6-05E15BBB10B3}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{D05DAFBC-1043-4587-8217-004B62E76A8C}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{D05DAFBC-1043-4587-8217-004B62E76A8C}"/>
   </bookViews>
   <sheets>
     <sheet name="turnover" sheetId="2" r:id="rId1"/>

</xml_diff>